<commit_message>
adding protein data and updated scripts
</commit_message>
<xml_diff>
--- a/RAnalysis/data/Physio_action_3_TOA_NUUROA_AIRBRUSH_trie_parT.xlsx
+++ b/RAnalysis/data/Physio_action_3_TOA_NUUROA_AIRBRUSH_trie_parT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hputnam/MyProjects/Toa_Nuuroa_transplant/RAnalysis/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E1AEA89-E2BB-5842-9535-43E1EA7FA417}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A9A94C-947F-CD49-BDE1-7C5A16BA21BD}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6980" yWindow="760" windowWidth="26820" windowHeight="18520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3420" yWindow="760" windowWidth="26820" windowHeight="18520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1849" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1859" uniqueCount="861">
   <si>
     <t>ID_microfragment</t>
   </si>
@@ -2593,6 +2593,24 @@
   </si>
   <si>
     <t>colony_id</t>
+  </si>
+  <si>
+    <t>SE25_T3_R1</t>
+  </si>
+  <si>
+    <t>SE25_T3_R2</t>
+  </si>
+  <si>
+    <t>SE25_T3_R3</t>
+  </si>
+  <si>
+    <t>SE25_T3_R4</t>
+  </si>
+  <si>
+    <t>SE25_T3_R5</t>
+  </si>
+  <si>
+    <t>changed t4 to t3 becasue of mislabel</t>
   </si>
 </sst>
 </file>
@@ -2794,7 +2812,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2824,11 +2842,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3052,7 +3079,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I2373"/>
+  <dimension ref="A1:K2373"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -12176,7 +12203,7 @@
         <v>1.23</v>
       </c>
     </row>
-    <row r="337" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A337" s="1" t="s">
         <v>615</v>
       </c>
@@ -12203,7 +12230,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="338" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A338" s="1" t="s">
         <v>617</v>
       </c>
@@ -12230,7 +12257,7 @@
         <v>7.84</v>
       </c>
     </row>
-    <row r="339" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A339" s="1" t="s">
         <v>619</v>
       </c>
@@ -12257,7 +12284,7 @@
         <v>8.06</v>
       </c>
     </row>
-    <row r="340" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A340" s="1" t="s">
         <v>621</v>
       </c>
@@ -12284,7 +12311,7 @@
         <v>0.89</v>
       </c>
     </row>
-    <row r="341" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A341" s="1" t="s">
         <v>623</v>
       </c>
@@ -12311,7 +12338,7 @@
         <v>0.91</v>
       </c>
     </row>
-    <row r="342" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A342" s="1" t="s">
         <v>625</v>
       </c>
@@ -12338,7 +12365,7 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="343" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A343" s="1" t="s">
         <v>627</v>
       </c>
@@ -12365,7 +12392,7 @@
         <v>7.42</v>
       </c>
     </row>
-    <row r="344" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A344" s="1" t="s">
         <v>629</v>
       </c>
@@ -12392,7 +12419,7 @@
         <v>8.61</v>
       </c>
     </row>
-    <row r="345" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A345" s="1" t="s">
         <v>631</v>
       </c>
@@ -12419,7 +12446,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="346" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A346" s="1" t="s">
         <v>633</v>
       </c>
@@ -12446,12 +12473,12 @@
         <v>8.26</v>
       </c>
     </row>
-    <row r="347" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A347" s="1" t="s">
         <v>635</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>636</v>
+        <v>855</v>
       </c>
       <c r="C347" s="1" t="s">
         <v>486</v>
@@ -12472,13 +12499,19 @@
       <c r="I347" s="12">
         <v>7.83</v>
       </c>
-    </row>
-    <row r="348" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J347" s="1" t="s">
+        <v>636</v>
+      </c>
+      <c r="K347" s="21" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="348" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A348" s="1" t="s">
         <v>637</v>
       </c>
       <c r="B348" s="1" t="s">
-        <v>638</v>
+        <v>856</v>
       </c>
       <c r="C348" s="1" t="s">
         <v>486</v>
@@ -12499,13 +12532,19 @@
       <c r="I348" s="12">
         <v>7.41</v>
       </c>
-    </row>
-    <row r="349" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J348" s="1" t="s">
+        <v>638</v>
+      </c>
+      <c r="K348" s="21" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="349" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A349" s="1" t="s">
         <v>639</v>
       </c>
       <c r="B349" s="1" t="s">
-        <v>640</v>
+        <v>857</v>
       </c>
       <c r="C349" s="1" t="s">
         <v>486</v>
@@ -12526,13 +12565,19 @@
       <c r="I349" s="12">
         <v>7.38</v>
       </c>
-    </row>
-    <row r="350" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J349" s="1" t="s">
+        <v>640</v>
+      </c>
+      <c r="K349" s="21" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="350" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A350" s="1" t="s">
         <v>641</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>642</v>
+        <v>858</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>486</v>
@@ -12553,13 +12598,19 @@
       <c r="I350" s="12">
         <v>8.0500000000000007</v>
       </c>
-    </row>
-    <row r="351" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J350" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="K350" s="21" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="351" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A351" s="1" t="s">
         <v>643</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>644</v>
+        <v>859</v>
       </c>
       <c r="C351" s="1" t="s">
         <v>486</v>
@@ -12580,8 +12631,14 @@
       <c r="I351" s="12">
         <v>8</v>
       </c>
-    </row>
-    <row r="352" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="J351" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="K351" s="21" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="352" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A352" s="1" t="s">
         <v>645</v>
       </c>
@@ -23089,8 +23146,13 @@
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <conditionalFormatting sqref="B1:B1001">
+    <cfRule type="notContainsBlanks" dxfId="1" priority="2">
+      <formula>LEN(TRIM(B1))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J347:J351">
     <cfRule type="notContainsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(B1))&gt;0</formula>
+      <formula>LEN(TRIM(J347))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>

</xml_diff>